<commit_message>
feat(admin/trades): template columns match Trades table + Excel-only upload
- Template/upload columns now mirror the Trades table exactly:
  USER, SYMBOL, SIDE, LOTS, OPEN, CURRENT, SPREAD, P&L, COMM., SL, TP, OPENED.
  Only USER/SYMBOL/SIDE/LOTS/OPEN/SL/TP are used; CURRENT/SPREAD/P&L/COMM./
  OPENED are display-only and ignored on upload.
- Upload now accepts ONLY .xlsx — frontend rejects other files with a warning,
  backend also enforces .xlsx and returns a clear error. Dropped CSV support.
- Regenerated dummy template with the new columns.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/trade_upload_template.xlsx
+++ b/docs/templates/trade_upload_template.xlsx
@@ -413,64 +413,82 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>user_email</t>
+          <t>USER</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>account_number</t>
+          <t>SYMBOL</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>symbol</t>
+          <t>SIDE</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>side</t>
+          <t>LOTS</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>lots</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>open_price</t>
+          <t>CURRENT</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>stop_loss</t>
+          <t>SPREAD</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>take_profit</t>
+          <t>P&amp;L</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>comment</t>
+          <t>COMM.</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>OPENED</t>
         </is>
       </c>
     </row>
@@ -480,32 +498,31 @@
           <t>trader@example.com</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>XAUUSD</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
           <t>buy</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="D2" t="n">
         <v>0.1</v>
       </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="n">
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="n">
         <v>4750</v>
       </c>
-      <c r="H2" t="n">
+      <c r="K2" t="n">
         <v>4850</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Example market buy</t>
-        </is>
-      </c>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -515,36 +532,31 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>100245</t>
+          <t>EURUSD</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>EURUSD</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
           <t>sell</t>
         </is>
       </c>
+      <c r="D3" t="n">
+        <v>0.05</v>
+      </c>
       <c r="E3" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="F3" t="n">
         <v>1.085</v>
       </c>
-      <c r="G3" t="n">
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="n">
         <v>1.09</v>
       </c>
-      <c r="H3" t="n">
+      <c r="K3" t="n">
         <v>1.08</v>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Example with entry price</t>
-        </is>
-      </c>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -552,28 +564,27 @@
           <t>hari@example.com</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BTCUSD</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BTCUSD</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
           <t>buy</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="D4" t="n">
         <v>0.01</v>
       </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Market buy, no SL/TP</t>
-        </is>
-      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(admin/trades): make upload template placeholders obvious + clearer 'user not found'
The template shipped with example emails (trader@example.com) that don't
exist, so uploading it unchanged failed with 'user not found'. Replace the
placeholder with 'REPLACE-WITH-REAL-USER-EMAIL' so it's obvious the USER
column must be a real registered email, and make the row error actionable.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/trade_upload_template.xlsx
+++ b/docs/templates/trade_upload_template.xlsx
@@ -413,10 +413,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -495,7 +495,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>trader@example.com</t>
+          <t>REPLACE-WITH-REAL-USER-EMAIL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>trader@example.com</t>
+          <t>REPLACE-WITH-REAL-USER-EMAIL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -558,34 +558,6 @@
       </c>
       <c r="L3" t="inlineStr"/>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>hari@example.com</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>BTCUSD</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>buy</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(admin/trades): auto-create dummy user for unknown emails on upload
If a row's USER email isn't a registered user, provision a demo (dummy)
user + trading account (is_demo, 'DM' account number) so the trade still
shows in the Trades list. Registered users keep using their real account.
Result summary now reports dummy_users_created; template uses demo emails
with example prices so it works out of the box.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/trade_upload_template.xlsx
+++ b/docs/templates/trade_upload_template.xlsx
@@ -416,7 +416,7 @@
   <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -495,7 +495,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>REPLACE-WITH-REAL-USER-EMAIL</t>
+          <t>dummy1@demo.com</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -511,23 +511,25 @@
       <c r="D2" t="n">
         <v>0.1</v>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>4100</v>
+      </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="n">
-        <v>4750</v>
+        <v>4000</v>
       </c>
       <c r="K2" t="n">
-        <v>4850</v>
+        <v>4200</v>
       </c>
       <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>REPLACE-WITH-REAL-USER-EMAIL</t>
+          <t>dummy2@demo.com</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">

</xml_diff>

<commit_message>
feat(admin/trades): show the exact USER name from Excel in the Trades list
Add user_name to Position/Order/History outputs (from the user's first+last
name) and display user_name || user_email in the Trades table + detail modals.
Uploaded rows whose USER isn't a registered email now show the typed value
verbatim (the demo user's name = the Excel value). Template examples use
names (Rahul Sharma / Priya Verma); result label reads 'New users'.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/trade_upload_template.xlsx
+++ b/docs/templates/trade_upload_template.xlsx
@@ -416,7 +416,7 @@
   <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -495,7 +495,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>dummy1@demo.com</t>
+          <t>Rahul Sharma</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -529,7 +529,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>dummy2@demo.com</t>
+          <t>Priya Verma</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">

</xml_diff>